<commit_message>
More appendix cleaning up
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/kiribati_tb_modelling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3511CEF-02A0-E249-B44D-A8105751CA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A75837-202D-A442-810F-0CA8413A4090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="38400" yWindow="3240" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>
@@ -252,9 +252,6 @@
     <t>Rel. susceptibility to infection for under 15 year-old individuals (ref. 15 and over)</t>
   </si>
   <si>
-    <t>Rel. infectiousness of subclinical TB (ref. clinical TB)</t>
-  </si>
-  <si>
     <t>Rel. infectiousness of 'less infectious' TB (ref. 'more infectious' TB)</t>
   </si>
   <si>
@@ -264,36 +261,9 @@
     <t>Annual rate of TB detection in 2020</t>
   </si>
   <si>
-    <t>Probability PEARL-positive for 'subclinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability PEARL-positive for 'clinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability PEARL-positive for 'subclinical' and 'more infectious' category</t>
-  </si>
-  <si>
-    <t>Probability PEARL-positive for 'clinical' and 'more infectious' category</t>
-  </si>
-  <si>
     <t>TPT completion percentage</t>
   </si>
   <si>
-    <t>Probability CXR-positive for 'subclinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability CXR-positive for 'clinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability CXR-positive for 'subclinical' and 'more infectious' category</t>
-  </si>
-  <si>
-    <t>Probability CXR-positive for 'clinical' and 'more infectious' category</t>
-  </si>
-  <si>
-    <t>Relative detection rate of subclinical TB under passive case finding (ref. clinical TB)</t>
-  </si>
-  <si>
     <t>prev_se_subclin_lowinf_plts</t>
   </si>
   <si>
@@ -306,18 +276,6 @@
     <t>prev_se_clin_inf_plts</t>
   </si>
   <si>
-    <t>Probability PLTS-positive for 'subclinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability PLTS-positive for 'clinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability PLTS-positive for 'subclinical' and 'more infectious' category</t>
-  </si>
-  <si>
-    <t>Probability PLTS-positive for 'clinical' and 'more infectious' category</t>
-  </si>
-  <si>
     <t>prev_se_subclin_lowinf_ssx</t>
   </si>
   <si>
@@ -330,18 +288,6 @@
     <t>prev_se_clin_inf_ssx</t>
   </si>
   <si>
-    <t>Probability SSx-positive for 'subclinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability SSx-positive for 'clinical' and 'less infectious' category</t>
-  </si>
-  <si>
-    <t>Probability SSx-positive for 'subclinical' and 'more infectious' category</t>
-  </si>
-  <si>
-    <t>Probability SSx-positive for 'clinical' and 'more infectious' category</t>
-  </si>
-  <si>
     <t>passive_detection_inflection</t>
   </si>
   <si>
@@ -417,21 +363,9 @@
     <t>Average TB treatment duration (years)</t>
   </si>
   <si>
-    <t>Rate of self-recovery for subclinical TB (/year)</t>
-  </si>
-  <si>
-    <t>Rate of TB mortality for 'less infectious' clinical disease (/year)</t>
-  </si>
-  <si>
-    <t>Rate of TB mortality for 'more infectious' clinical disease (/year)</t>
-  </si>
-  <si>
     <t>Rate of progression from 'less infectious' to 'more infectious' TB (/year)</t>
   </si>
   <si>
-    <t>Rate of progression from subclinical to clinical TB (/year)</t>
-  </si>
-  <si>
     <t>Rate of transition from 'contained' to 'cleared' (all ages, /year)</t>
   </si>
   <si>
@@ -462,9 +396,6 @@
     <t>Rel. risk of reinfection from 'cleared' and 'recovered' compartment (ref. 'mtb-naïve')</t>
   </si>
   <si>
-    <t>Rate of regression from clinical to subclinical TB (/year)</t>
-  </si>
-  <si>
     <t>Rate of regression from 'more infectious' to 'less infectious' TB (/year)</t>
   </si>
   <si>
@@ -478,6 +409,75 @@
   </si>
   <si>
     <t>Relative susceptibility to infection of hard-to-reach population (ref. screening-reachable)</t>
+  </si>
+  <si>
+    <t>Rate of progression from asymptomatic to symptomatic TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of regression from symptomatic to asymptomatic TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of TB mortality for 'more infectious' symptomatic disease (/year)</t>
+  </si>
+  <si>
+    <t>Rate of TB mortality for 'less infectious' symptomatic disease (/year)</t>
+  </si>
+  <si>
+    <t>Rate of self-recovery for asymptomatic TB (/year)</t>
+  </si>
+  <si>
+    <t>Probability PEARL-positive for 'asymptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PEARL-positive for 'symptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PEARL-positive for 'asymptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PEARL-positive for 'symptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PLTS-positive for 'asymptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PLTS-positive for 'symptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PLTS-positive for 'asymptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability PLTS-positive for 'symptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability CXR-positive for 'asymptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability CXR-positive for 'symptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability CXR-positive for 'asymptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability CXR-positive for 'symptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability SSx-positive for 'asymptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability SSx-positive for 'symptomatic' and 'less infectious' category</t>
+  </si>
+  <si>
+    <t>Probability SSx-positive for 'asymptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Probability SSx-positive for 'symptomatic' and 'more infectious' category</t>
+  </si>
+  <si>
+    <t>Relative detection rate of asymptomatic TB under passive case finding (ref. symptomatic TB)</t>
+  </si>
+  <si>
+    <t>Rel. infectiousness of asymptomatic TB (ref. symptomatic TB)</t>
   </si>
 </sst>
 </file>
@@ -988,7 +988,7 @@
         <v>24</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1016,7 +1016,7 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="B3" s="2">
         <v>0.05</v>
@@ -1031,12 +1031,12 @@
         <v>0.05</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1051,7 +1051,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>28</v>
@@ -1059,7 +1059,7 @@
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="B5" s="2">
         <v>0.2</v>
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>29</v>
@@ -1120,7 +1120,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>31</v>
@@ -1157,7 +1157,7 @@
         <v>0.5</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>71</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1168,7 +1168,7 @@
         <v>0.4</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -1182,7 +1182,7 @@
         <v>2.4</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>34</v>
@@ -1199,7 +1199,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>137</v>
+        <v>115</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>25</v>
@@ -1213,7 +1213,7 @@
         <v>0.1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -1227,10 +1227,10 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -1241,7 +1241,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>35</v>
@@ -1258,7 +1258,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
@@ -1272,7 +1272,7 @@
         <v>2</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
@@ -1295,7 +1295,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>36</v>
@@ -1321,7 +1321,7 @@
         <v>0.1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>39</v>
@@ -1347,7 +1347,7 @@
         <v>5</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>40</v>
@@ -1364,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>41</v>
@@ -1390,7 +1390,7 @@
         <v>10</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>42</v>
@@ -1407,7 +1407,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>142</v>
+        <v>119</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>43</v>
@@ -1424,7 +1424,7 @@
         <v>0.38900000000000001</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>38</v>
@@ -1458,7 +1458,7 @@
         <v>0.4</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>37</v>
@@ -1484,7 +1484,7 @@
         <v>5</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>25</v>
@@ -1498,7 +1498,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>48</v>
@@ -1515,7 +1515,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>44</v>
@@ -1523,29 +1523,29 @@
     </row>
     <row r="30" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="B30" s="5">
         <v>0.75</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="B31" s="5">
         <v>0.75</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B32" s="5">
         <v>0.35</v>
@@ -1560,7 +1560,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1571,7 +1571,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>75</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1582,7 +1582,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>76</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>77</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1604,63 +1604,63 @@
         <v>1</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>78</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B37" s="10">
         <v>0.3</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>89</v>
+        <v>133</v>
       </c>
       <c r="J37" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B38" s="10">
         <v>1</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>90</v>
+        <v>134</v>
       </c>
       <c r="J38" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B39" s="10">
         <v>0.5</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>91</v>
+        <v>135</v>
       </c>
       <c r="J39" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="40" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B40" s="10">
         <v>1</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>92</v>
+        <v>136</v>
       </c>
       <c r="J40" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1680,7 +1680,7 @@
         <v>0.52</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>80</v>
+        <v>137</v>
       </c>
     </row>
     <row r="42" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1691,7 +1691,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>81</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1711,7 +1711,7 @@
         <v>0.93</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>82</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1722,51 +1722,51 @@
         <v>1</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>83</v>
+        <v>140</v>
       </c>
     </row>
     <row r="45" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="B45" s="12">
         <v>0</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="B46" s="12">
         <v>1</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>98</v>
+        <v>142</v>
       </c>
     </row>
     <row r="47" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B47" s="12">
         <v>0</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>99</v>
+        <v>143</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="B48" s="12">
         <v>1</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>100</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -1777,7 +1777,7 @@
         <v>70</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>44</v>
@@ -1791,15 +1791,15 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>84</v>
+        <v>145</v>
       </c>
       <c r="J50" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="B51" s="13">
         <v>2000</v>
@@ -1814,23 +1814,23 @@
         <v>2020</v>
       </c>
       <c r="G51" s="13" t="s">
-        <v>144</v>
+        <v>121</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="B52" s="13">
         <v>0.15</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="B53">
         <v>0.5</v>
@@ -1845,12 +1845,12 @@
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="B54">
         <v>0.5</v>
@@ -1865,40 +1865,40 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>139</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B55">
         <v>0.85</v>
       </c>
       <c r="G55" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="B56">
         <v>0.5</v>
       </c>
       <c r="G56" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="B57">
         <v>1.5</v>
       </c>
       <c r="G57" t="s">
-        <v>146</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>